<commit_message>
refactor: Update Excel mappings and remove value calculations
- Target the "Pozycje otwarte" sheet.
- Update `ASSET_MAPPING` to match precise asset rows (MSFT: 16, GOOGL: 17, TSLA: 24, BTC/USDT: 25).
- Write the current date (YYYY-MM-DD) to column 'A' and the current price to column 'G'.
- Remove the volume variables and notional/liability PnL calculation logic.
- Fix docstring in `main.py` and ensure `__pycache__` is excluded.

Co-authored-by: JoziMate <69837976+JoziMate@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Dziennik_inwestora.xlsx
+++ b/Dziennik_inwestora.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="v2 (Instytucjonalna)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pozycje otwarte" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,76 +413,84 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A15:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Asset</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Current Price</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Current Value</t>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Data aktualizacji</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Instrument</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Cena bieżąca</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>MSFT</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="G16" t="n">
         <v>405.2099914550781</v>
       </c>
-      <c r="C2" t="n">
-        <v>405.2099914550781</v>
-      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>GOOGL</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="G17" t="n">
         <v>402.6199951171875</v>
       </c>
-      <c r="C3" t="n">
-        <v>402.6199951171875</v>
-      </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>TSLA</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="G24" t="n">
         <v>445.2699890136719</v>
       </c>
-      <c r="C4" t="n">
-        <v>22263.49945068359</v>
-      </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>BTC/USDT</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>79395.99000000001</v>
-      </c>
-      <c r="C5" t="n">
-        <v>158791.98</v>
+      <c r="G25" t="n">
+        <v>79745.71000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>